<commit_message>
Update Steam sale data
</commit_message>
<xml_diff>
--- a/steam_sales_output/publisher_sales.xlsx
+++ b/steam_sales_output/publisher_sales.xlsx
@@ -3346,12 +3346,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -3372,7 +3372,7 @@
         </is>
       </c>
       <c r="H45" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -3413,12 +3413,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="F46" t="n">
@@ -3430,7 +3430,7 @@
         </is>
       </c>
       <c r="H46" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -15385,12 +15385,12 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="H114" s="2" t="inlineStr">
@@ -18395,12 +18395,12 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -37482,12 +37482,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -37508,7 +37508,7 @@
         </is>
       </c>
       <c r="H22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -37549,12 +37549,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -37566,7 +37566,7 @@
         </is>
       </c>
       <c r="H23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>

</xml_diff>